<commit_message>
feat(universe): execute world-difficulty partition S36
</commit_message>
<xml_diff>
--- a/config/data/AiGraph.xlsx
+++ b/config/data/AiGraph.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -766,6 +766,1139 @@
         <v>8</v>
       </c>
     </row>
+    <row r="25">
+      <c r="B25" t="n">
+        <v>980010</v>
+      </c>
+      <c r="C25" t="n">
+        <v>980701</v>
+      </c>
+      <c r="D25" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="n">
+        <v>980011</v>
+      </c>
+      <c r="C26" t="n">
+        <v>980706</v>
+      </c>
+      <c r="D26" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="n">
+        <v>980012</v>
+      </c>
+      <c r="C27" t="n">
+        <v>980711</v>
+      </c>
+      <c r="D27" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="n">
+        <v>990010</v>
+      </c>
+      <c r="C28" t="n">
+        <v>990701</v>
+      </c>
+      <c r="D28" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="n">
+        <v>990011</v>
+      </c>
+      <c r="C29" t="n">
+        <v>990704</v>
+      </c>
+      <c r="D29" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="n">
+        <v>990012</v>
+      </c>
+      <c r="C30" t="n">
+        <v>990707</v>
+      </c>
+      <c r="D30" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="n">
+        <v>1000010</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1000701</v>
+      </c>
+      <c r="D31" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="n">
+        <v>1000011</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1000706</v>
+      </c>
+      <c r="D32" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="n">
+        <v>1010010</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1010701</v>
+      </c>
+      <c r="D33" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="n">
+        <v>1020010</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1020701</v>
+      </c>
+      <c r="D34" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="n">
+        <v>1020011</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1020705</v>
+      </c>
+      <c r="D35" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="n">
+        <v>1020012</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1020711</v>
+      </c>
+      <c r="D36" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="n">
+        <v>1030010</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1030701</v>
+      </c>
+      <c r="D37" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="n">
+        <v>1030011</v>
+      </c>
+      <c r="C38" t="n">
+        <v>1030704</v>
+      </c>
+      <c r="D38" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="n">
+        <v>1030012</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1030710</v>
+      </c>
+      <c r="D39" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="n">
+        <v>1040010</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1040701</v>
+      </c>
+      <c r="D40" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="n">
+        <v>1040011</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1040705</v>
+      </c>
+      <c r="D41" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="n">
+        <v>1040012</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1040715</v>
+      </c>
+      <c r="D42" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="n">
+        <v>1050010</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1050701</v>
+      </c>
+      <c r="D43" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="n">
+        <v>1060010</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1060701</v>
+      </c>
+      <c r="D44" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="n">
+        <v>1060011</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1060721</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="n">
+        <v>1060012</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1060741</v>
+      </c>
+      <c r="D46" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="n">
+        <v>1070010</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1070701</v>
+      </c>
+      <c r="D47" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="n">
+        <v>1070011</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1070705</v>
+      </c>
+      <c r="D48" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="n">
+        <v>1070012</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1070709</v>
+      </c>
+      <c r="D49" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="n">
+        <v>1080010</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1080701</v>
+      </c>
+      <c r="D50" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="n">
+        <v>1080011</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1080705</v>
+      </c>
+      <c r="D51" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="n">
+        <v>1080012</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1080710</v>
+      </c>
+      <c r="D52" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="n">
+        <v>1090041</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1094101</v>
+      </c>
+      <c r="D53" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="n">
+        <v>1090042</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1094102</v>
+      </c>
+      <c r="D54" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="n">
+        <v>1090043</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1094106</v>
+      </c>
+      <c r="D55" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="n">
+        <v>1090044</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1094110</v>
+      </c>
+      <c r="D56" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="n">
+        <v>1090045</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1094112</v>
+      </c>
+      <c r="D57" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="n">
+        <v>1090046</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1094113</v>
+      </c>
+      <c r="D58" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="n">
+        <v>1090047</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1094116</v>
+      </c>
+      <c r="D59" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="n">
+        <v>1090048</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1094122</v>
+      </c>
+      <c r="D60" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="n">
+        <v>1090049</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1094126</v>
+      </c>
+      <c r="D61" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="n">
+        <v>1090050</v>
+      </c>
+      <c r="C62" t="n">
+        <v>1094127</v>
+      </c>
+      <c r="D62" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="n">
+        <v>1090051</v>
+      </c>
+      <c r="C63" t="n">
+        <v>1094131</v>
+      </c>
+      <c r="D63" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="n">
+        <v>1090052</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1094136</v>
+      </c>
+      <c r="D64" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="n">
+        <v>1100041</v>
+      </c>
+      <c r="C65" t="n">
+        <v>1104101</v>
+      </c>
+      <c r="D65" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="n">
+        <v>1100042</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1104104</v>
+      </c>
+      <c r="D66" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="n">
+        <v>1100043</v>
+      </c>
+      <c r="C67" t="n">
+        <v>1104105</v>
+      </c>
+      <c r="D67" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="n">
+        <v>1100044</v>
+      </c>
+      <c r="C68" t="n">
+        <v>1104107</v>
+      </c>
+      <c r="D68" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="n">
+        <v>1100045</v>
+      </c>
+      <c r="C69" t="n">
+        <v>1104111</v>
+      </c>
+      <c r="D69" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="n">
+        <v>1100046</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1104112</v>
+      </c>
+      <c r="D70" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="n">
+        <v>1100047</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1104114</v>
+      </c>
+      <c r="D71" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="n">
+        <v>1100048</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1104118</v>
+      </c>
+      <c r="D72" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="n">
+        <v>1100049</v>
+      </c>
+      <c r="C73" t="n">
+        <v>1104122</v>
+      </c>
+      <c r="D73" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="n">
+        <v>1100050</v>
+      </c>
+      <c r="C74" t="n">
+        <v>1104127</v>
+      </c>
+      <c r="D74" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="n">
+        <v>1100051</v>
+      </c>
+      <c r="C75" t="n">
+        <v>1104132</v>
+      </c>
+      <c r="D75" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="n">
+        <v>1100052</v>
+      </c>
+      <c r="C76" t="n">
+        <v>1104133</v>
+      </c>
+      <c r="D76" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="n">
+        <v>1110041</v>
+      </c>
+      <c r="C77" t="n">
+        <v>1114101</v>
+      </c>
+      <c r="D77" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="n">
+        <v>1110042</v>
+      </c>
+      <c r="C78" t="n">
+        <v>1114104</v>
+      </c>
+      <c r="D78" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="n">
+        <v>1110043</v>
+      </c>
+      <c r="C79" t="n">
+        <v>1114105</v>
+      </c>
+      <c r="D79" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="n">
+        <v>1110044</v>
+      </c>
+      <c r="C80" t="n">
+        <v>1114109</v>
+      </c>
+      <c r="D80" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="n">
+        <v>1110045</v>
+      </c>
+      <c r="C81" t="n">
+        <v>1114113</v>
+      </c>
+      <c r="D81" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" t="n">
+        <v>1110046</v>
+      </c>
+      <c r="C82" t="n">
+        <v>1114116</v>
+      </c>
+      <c r="D82" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" t="n">
+        <v>1110047</v>
+      </c>
+      <c r="C83" t="n">
+        <v>1114117</v>
+      </c>
+      <c r="D83" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" t="n">
+        <v>1110048</v>
+      </c>
+      <c r="C84" t="n">
+        <v>1114118</v>
+      </c>
+      <c r="D84" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" t="n">
+        <v>1110049</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1114119</v>
+      </c>
+      <c r="D85" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" t="n">
+        <v>1110050</v>
+      </c>
+      <c r="C86" t="n">
+        <v>1114120</v>
+      </c>
+      <c r="D86" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" t="n">
+        <v>1110051</v>
+      </c>
+      <c r="C87" t="n">
+        <v>1114121</v>
+      </c>
+      <c r="D87" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" t="n">
+        <v>1110052</v>
+      </c>
+      <c r="C88" t="n">
+        <v>1114126</v>
+      </c>
+      <c r="D88" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" t="n">
+        <v>1120041</v>
+      </c>
+      <c r="C89" t="n">
+        <v>1124101</v>
+      </c>
+      <c r="D89" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" t="n">
+        <v>1120042</v>
+      </c>
+      <c r="C90" t="n">
+        <v>1124102</v>
+      </c>
+      <c r="D90" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" t="n">
+        <v>1120043</v>
+      </c>
+      <c r="C91" t="n">
+        <v>1124103</v>
+      </c>
+      <c r="D91" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" t="n">
+        <v>1120044</v>
+      </c>
+      <c r="C92" t="n">
+        <v>1124110</v>
+      </c>
+      <c r="D92" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" t="n">
+        <v>1120045</v>
+      </c>
+      <c r="C93" t="n">
+        <v>1124113</v>
+      </c>
+      <c r="D93" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" t="n">
+        <v>1120046</v>
+      </c>
+      <c r="C94" t="n">
+        <v>1124114</v>
+      </c>
+      <c r="D94" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" t="n">
+        <v>1120047</v>
+      </c>
+      <c r="C95" t="n">
+        <v>1124116</v>
+      </c>
+      <c r="D95" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" t="n">
+        <v>1120048</v>
+      </c>
+      <c r="C96" t="n">
+        <v>1124118</v>
+      </c>
+      <c r="D96" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" t="n">
+        <v>1120049</v>
+      </c>
+      <c r="C97" t="n">
+        <v>1124119</v>
+      </c>
+      <c r="D97" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" t="n">
+        <v>1120050</v>
+      </c>
+      <c r="C98" t="n">
+        <v>1124120</v>
+      </c>
+      <c r="D98" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" t="n">
+        <v>1120051</v>
+      </c>
+      <c r="C99" t="n">
+        <v>1124122</v>
+      </c>
+      <c r="D99" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" t="n">
+        <v>1120052</v>
+      </c>
+      <c r="C100" t="n">
+        <v>1124123</v>
+      </c>
+      <c r="D100" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" t="n">
+        <v>1130041</v>
+      </c>
+      <c r="C101" t="n">
+        <v>1134101</v>
+      </c>
+      <c r="D101" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" t="n">
+        <v>1130042</v>
+      </c>
+      <c r="C102" t="n">
+        <v>1134105</v>
+      </c>
+      <c r="D102" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" t="n">
+        <v>1130043</v>
+      </c>
+      <c r="C103" t="n">
+        <v>1134106</v>
+      </c>
+      <c r="D103" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" t="n">
+        <v>1130044</v>
+      </c>
+      <c r="C104" t="n">
+        <v>1134110</v>
+      </c>
+      <c r="D104" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" t="n">
+        <v>1130045</v>
+      </c>
+      <c r="C105" t="n">
+        <v>1134114</v>
+      </c>
+      <c r="D105" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" t="n">
+        <v>1130046</v>
+      </c>
+      <c r="C106" t="n">
+        <v>1134118</v>
+      </c>
+      <c r="D106" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" t="n">
+        <v>1130047</v>
+      </c>
+      <c r="C107" t="n">
+        <v>1134120</v>
+      </c>
+      <c r="D107" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" t="n">
+        <v>1130048</v>
+      </c>
+      <c r="C108" t="n">
+        <v>1134121</v>
+      </c>
+      <c r="D108" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" t="n">
+        <v>1130049</v>
+      </c>
+      <c r="C109" t="n">
+        <v>1134125</v>
+      </c>
+      <c r="D109" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" t="n">
+        <v>1130050</v>
+      </c>
+      <c r="C110" t="n">
+        <v>1134126</v>
+      </c>
+      <c r="D110" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" t="n">
+        <v>1130051</v>
+      </c>
+      <c r="C111" t="n">
+        <v>1134130</v>
+      </c>
+      <c r="D111" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" t="n">
+        <v>1130052</v>
+      </c>
+      <c r="C112" t="n">
+        <v>1134134</v>
+      </c>
+      <c r="D112" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" t="n">
+        <v>1140041</v>
+      </c>
+      <c r="C113" t="n">
+        <v>1144101</v>
+      </c>
+      <c r="D113" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" t="n">
+        <v>1140042</v>
+      </c>
+      <c r="C114" t="n">
+        <v>1144102</v>
+      </c>
+      <c r="D114" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" t="n">
+        <v>1140043</v>
+      </c>
+      <c r="C115" t="n">
+        <v>1144105</v>
+      </c>
+      <c r="D115" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" t="n">
+        <v>1140044</v>
+      </c>
+      <c r="C116" t="n">
+        <v>1144108</v>
+      </c>
+      <c r="D116" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" t="n">
+        <v>1140045</v>
+      </c>
+      <c r="C117" t="n">
+        <v>1144111</v>
+      </c>
+      <c r="D117" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" t="n">
+        <v>1140046</v>
+      </c>
+      <c r="C118" t="n">
+        <v>1144114</v>
+      </c>
+      <c r="D118" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" t="n">
+        <v>1140047</v>
+      </c>
+      <c r="C119" t="n">
+        <v>1144117</v>
+      </c>
+      <c r="D119" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" t="n">
+        <v>1140048</v>
+      </c>
+      <c r="C120" t="n">
+        <v>1144120</v>
+      </c>
+      <c r="D120" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" t="n">
+        <v>1140049</v>
+      </c>
+      <c r="C121" t="n">
+        <v>1144122</v>
+      </c>
+      <c r="D121" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" t="n">
+        <v>1140050</v>
+      </c>
+      <c r="C122" t="n">
+        <v>1144124</v>
+      </c>
+      <c r="D122" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" t="n">
+        <v>1140051</v>
+      </c>
+      <c r="C123" t="n">
+        <v>1144126</v>
+      </c>
+      <c r="D123" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" t="n">
+        <v>1140052</v>
+      </c>
+      <c r="C124" t="n">
+        <v>1144128</v>
+      </c>
+      <c r="D124" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" t="n">
+        <v>1150041</v>
+      </c>
+      <c r="C125" t="n">
+        <v>1154101</v>
+      </c>
+      <c r="D125" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" t="n">
+        <v>1150042</v>
+      </c>
+      <c r="C126" t="n">
+        <v>1154106</v>
+      </c>
+      <c r="D126" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" t="n">
+        <v>1150043</v>
+      </c>
+      <c r="C127" t="n">
+        <v>1154107</v>
+      </c>
+      <c r="D127" t="n">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>